<commit_message>
feat: Add active policy list and guide banners for admin and B2C
</commit_message>
<xml_diff>
--- a/insurance_data/3_family/child/extracted_data.xlsx
+++ b/insurance_data/3_family/child/extracted_data.xlsx
@@ -686,7 +686,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>1000만원 원</t>
+          <t>1000만원  원</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -707,7 +707,7 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t>file_16.xls</t>
+          <t>보장성_상품비교_20260608162103272.xls</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -742,7 +742,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>1000만원 원</t>
+          <t>1000만원  원</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -822,7 +822,7 @@
       </c>
       <c r="AM2" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="AN2" t="inlineStr">
@@ -879,7 +879,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>1000만원 원</t>
+          <t>1000만원  원</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -900,7 +900,7 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
-          <t>file_16.xls</t>
+          <t>보장성_상품비교_20260608162103272.xls</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>1000만원 원</t>
+          <t>1000만원  원</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
@@ -1015,7 +1015,7 @@
       </c>
       <c r="AM3" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="AN3" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>1000만원 원</t>
+          <t>1000만원  원</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1093,7 +1093,7 @@
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr">
         <is>
-          <t>file_16.xls</t>
+          <t>보장성_상품비교_20260608162103272.xls</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>1000만원 원</t>
+          <t>1000만원  원</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
@@ -1188,7 +1188,7 @@
       </c>
       <c r="AI4" t="inlineStr">
         <is>
-          <t>무해지/저해지환급</t>
+          <t>순수보장형</t>
         </is>
       </c>
       <c r="AJ4" t="inlineStr">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="AM4" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="AN4" t="inlineStr">
@@ -1265,7 +1265,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>1000만원 원</t>
+          <t>1000만원  원</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1286,7 +1286,7 @@
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
         <is>
-          <t>file_16.xls</t>
+          <t>보장성_상품비교_20260608162103272.xls</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -1321,7 +1321,7 @@
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>1000만원 원</t>
+          <t>1000만원  원</t>
         </is>
       </c>
       <c r="X5" t="inlineStr">
@@ -1381,7 +1381,7 @@
       </c>
       <c r="AI5" t="inlineStr">
         <is>
-          <t>무해지/저해지환급</t>
+          <t>순수보장형</t>
         </is>
       </c>
       <c r="AJ5" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="AM5" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="AN5" t="inlineStr">
@@ -1458,7 +1458,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>3000만원 원</t>
+          <t>3000만원  원</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1479,7 +1479,7 @@
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr">
         <is>
-          <t>file_16.xls</t>
+          <t>보장성_상품비교_20260608162103272.xls</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -1514,7 +1514,7 @@
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>3000만원 원</t>
+          <t>3000만원  원</t>
         </is>
       </c>
       <c r="X6" t="inlineStr">
@@ -1651,7 +1651,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>3000만원 원</t>
+          <t>3000만원  원</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1672,7 +1672,7 @@
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
         <is>
-          <t>file_16.xls</t>
+          <t>보장성_상품비교_20260608162103272.xls</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -1707,7 +1707,7 @@
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>3000만원 원</t>
+          <t>3000만원  원</t>
         </is>
       </c>
       <c r="X7" t="inlineStr">
@@ -1819,7 +1819,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>(무)다이렉트자녀보험2601(CM)</t>
+          <t>(무)다이렉트자녀보험2605(CM)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1865,7 +1865,7 @@
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
         <is>
-          <t>file_43.xls</t>
+          <t>장기보장성 비교 공시 (3).xls</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr"/>
@@ -1876,7 +1876,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>(무)다이렉트자녀보험2601(CM)</t>
+          <t>(무)다이렉트자녀보험2605(CM)</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -1948,7 +1948,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>(무)아이(I)러브(LOVE)플러스건강보험2601(10종)</t>
+          <t>(무)아이(I)러브(LOVE)플러스건강보험2604(10종)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1994,7 +1994,7 @@
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr">
         <is>
-          <t>file_43.xls</t>
+          <t>장기보장성 비교 공시 (3).xls</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr"/>
@@ -2005,7 +2005,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>(무)아이(I)러브(LOVE)플러스건강보험2601(10종)</t>
+          <t>(무)아이(I)러브(LOVE)플러스건강보험2604(10종)</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -2077,7 +2077,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>(무)아이(I)러브(LOVE)플러스건강보험2601(11종)</t>
+          <t>(무)아이(I)러브(LOVE)플러스건강보험2604(11종)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -2123,7 +2123,7 @@
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr">
         <is>
-          <t>file_43.xls</t>
+          <t>장기보장성 비교 공시 (3).xls</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr"/>
@@ -2134,7 +2134,7 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>(무)아이(I)러브(LOVE)플러스건강보험2601(11종)</t>
+          <t>(무)아이(I)러브(LOVE)플러스건강보험2604(11종)</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -2206,7 +2206,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>(무)아이(I)러브(LOVE)플러스건강보험2601(2종)</t>
+          <t>(무)아이(I)러브(LOVE)플러스건강보험2604(2종)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -2252,7 +2252,7 @@
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr">
         <is>
-          <t>file_43.xls</t>
+          <t>장기보장성 비교 공시 (3).xls</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr"/>
@@ -2263,7 +2263,7 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>(무)아이(I)러브(LOVE)플러스건강보험2601(2종)</t>
+          <t>(무)아이(I)러브(LOVE)플러스건강보험2604(2종)</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>(무)아이(I)러브(LOVE)플러스건강보험2601(4종)</t>
+          <t>(무)아이(I)러브(LOVE)플러스건강보험2604(4종)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2381,7 +2381,7 @@
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr">
         <is>
-          <t>file_43.xls</t>
+          <t>장기보장성 비교 공시 (3).xls</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr"/>
@@ -2392,7 +2392,7 @@
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>(무)아이(I)러브(LOVE)플러스건강보험2601(4종)</t>
+          <t>(무)아이(I)러브(LOVE)플러스건강보험2604(4종)</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
@@ -2464,7 +2464,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>(무)아이(I)러브(LOVE)플러스건강보험2601(8종)</t>
+          <t>(무)아이(I)러브(LOVE)플러스건강보험2604(8종)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2510,7 +2510,7 @@
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr">
         <is>
-          <t>file_43.xls</t>
+          <t>장기보장성 비교 공시 (3).xls</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr"/>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>(무)아이(I)러브(LOVE)플러스건강보험2601(8종)</t>
+          <t>(무)아이(I)러브(LOVE)플러스건강보험2604(8종)</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
@@ -2593,7 +2593,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>(무)아이(I)러브(LOVE)플러스건강보험2601(9종)</t>
+          <t>(무)아이(I)러브(LOVE)플러스건강보험2604(9종)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2639,7 +2639,7 @@
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr">
         <is>
-          <t>file_43.xls</t>
+          <t>장기보장성 비교 공시 (3).xls</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr"/>
@@ -2650,7 +2650,7 @@
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>(무)아이(I)러브(LOVE)플러스건강보험2601(9종)</t>
+          <t>(무)아이(I)러브(LOVE)플러스건강보험2604(9종)</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
@@ -2768,7 +2768,7 @@
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr">
         <is>
-          <t>file_44.xls</t>
+          <t>장기보장성 비교 공시 (4).xls</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr"/>
@@ -2851,7 +2851,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>KB 금쪽같은 자녀보험Plus(무배당)(26.01)_1종 1형(자녀 납입면제 환급형)</t>
+          <t>KB 금쪽같은 자녀보험Plus(무배당)(26.04)_1종 1형(자녀 납입면제 환급형)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2897,7 +2897,7 @@
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr">
         <is>
-          <t>file_43.xls</t>
+          <t>장기보장성 비교 공시 (3).xls</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr"/>
@@ -2908,7 +2908,7 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>KB 금쪽같은 자녀보험Plus(무배당)(26.01)_1종 1형(자녀 납입면제 환급형)</t>
+          <t>KB 금쪽같은 자녀보험Plus(무배당)(26.04)_1종 1형(자녀 납입면제 환급형)</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
@@ -2980,7 +2980,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>KB 금쪽같은 자녀보험Plus(무배당)(26.01)_1종 2형(자녀 납입면제 기본형)</t>
+          <t>KB 금쪽같은 자녀보험Plus(무배당)(26.04)_1종 2형(자녀 납입면제 기본형)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -3026,7 +3026,7 @@
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr">
         <is>
-          <t>file_43.xls</t>
+          <t>장기보장성 비교 공시 (3).xls</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr"/>
@@ -3037,7 +3037,7 @@
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>KB 금쪽같은 자녀보험Plus(무배당)(26.01)_1종 2형(자녀 납입면제 기본형)</t>
+          <t>KB 금쪽같은 자녀보험Plus(무배당)(26.04)_1종 2형(자녀 납입면제 기본형)</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
@@ -3109,7 +3109,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>KB 금쪽같은 자녀보험Plus(무배당)(26.01)_2종(자녀 납입면제 표준형 해약환급금의 50‰지급형(납입기간 이후))</t>
+          <t>KB 금쪽같은 자녀보험Plus(무배당)(26.04)_2종(자녀 납입면제 표준형 해약환급금의 50‰지급형(납입기간 이후))</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -3155,7 +3155,7 @@
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr">
         <is>
-          <t>file_43.xls</t>
+          <t>장기보장성 비교 공시 (3).xls</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr"/>
@@ -3166,7 +3166,7 @@
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>KB 금쪽같은 자녀보험Plus(무배당)(26.01)_2종(자녀 납입면제 표준형 해약환급금의 50‰지급형(납입기간 이후))</t>
+          <t>KB 금쪽같은 자녀보험Plus(무배당)(26.04)_2종(자녀 납입면제 표준형 해약환급금의 50‰지급형(납입기간 이후))</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
@@ -3238,7 +3238,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>KB 다이렉트 자녀보험(무배당)(26.01)_1종</t>
+          <t>KB 다이렉트 자녀보험(무배당)(26.04)_1종</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -3284,7 +3284,7 @@
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr">
         <is>
-          <t>file_43.xls</t>
+          <t>장기보장성 비교 공시 (3).xls</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr"/>
@@ -3295,7 +3295,7 @@
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>KB 다이렉트 자녀보험(무배당)(26.01)_1종</t>
+          <t>KB 다이렉트 자녀보험(무배당)(26.04)_1종</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
@@ -3413,7 +3413,7 @@
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr">
         <is>
-          <t>file_43.xls</t>
+          <t>장기보장성 비교 공시 (3).xls</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr"/>
@@ -3542,7 +3542,7 @@
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr">
         <is>
-          <t>file_44.xls</t>
+          <t>장기보장성 비교 공시 (4).xls</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr"/>
@@ -3671,7 +3671,7 @@
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr">
         <is>
-          <t>file_16.xls</t>
+          <t>보장성_상품비교_20260608162103272.xls</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
@@ -3864,7 +3864,7 @@
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr">
         <is>
-          <t>file_16.xls</t>
+          <t>보장성_상품비교_20260608162103272.xls</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
@@ -3979,7 +3979,7 @@
       </c>
       <c r="AM23" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="AN23" t="inlineStr">
@@ -4057,7 +4057,7 @@
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr">
         <is>
-          <t>file_16.xls</t>
+          <t>보장성_상품비교_20260608162103272.xls</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
@@ -4172,7 +4172,7 @@
       </c>
       <c r="AM24" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="AN24" t="inlineStr">
@@ -4234,12 +4234,12 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>132,679 원</t>
+          <t>132,497 원</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>131,844 원</t>
+          <t>131,662 원</t>
         </is>
       </c>
       <c r="J25" t="inlineStr"/>
@@ -4250,7 +4250,7 @@
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr">
         <is>
-          <t>file_16.xls</t>
+          <t>보장성_상품비교_20260608162103272.xls</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
@@ -4290,12 +4290,12 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>40056  원</t>
+          <t>40000  원</t>
         </is>
       </c>
       <c r="Y25" t="inlineStr">
         <is>
-          <t>40,056  원</t>
+          <t>40,000  원</t>
         </is>
       </c>
       <c r="Z25" t="inlineStr">
@@ -4365,7 +4365,7 @@
       </c>
       <c r="AM25" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="AN25" t="inlineStr">
@@ -4397,7 +4397,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>(무)NH아이맘헤아림어린이보험[1종:해약환급금미지급형Ⅱ(납입중0‰,납입후50‰]2601</t>
+          <t>(무)NH아이맘헤아림어린이보험[1종:해약환급금미지급형Ⅱ(납입중0‰,납입후50‰]2604</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -4443,7 +4443,7 @@
       <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr">
         <is>
-          <t>file_43.xls</t>
+          <t>장기보장성 비교 공시 (3).xls</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr"/>
@@ -4454,7 +4454,7 @@
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>(무)NH아이맘헤아림어린이보험[1종:해약환급금미지급형Ⅱ(납입중0‰,납입후50‰]2601</t>
+          <t>(무)NH아이맘헤아림어린이보험[1종:해약환급금미지급형Ⅱ(납입중0‰,납입후50‰]2604</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
@@ -4526,7 +4526,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>(무)NH아이맘헤아림어린이보험[2종:표준형]2601</t>
+          <t>(무)NH아이맘헤아림어린이보험[2종:표준형]2604</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -4572,7 +4572,7 @@
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr">
         <is>
-          <t>file_43.xls</t>
+          <t>장기보장성 비교 공시 (3).xls</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr"/>
@@ -4583,7 +4583,7 @@
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>(무)NH아이맘헤아림어린이보험[2종:표준형]2601</t>
+          <t>(무)NH아이맘헤아림어린이보험[2종:표준형]2604</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
@@ -4701,7 +4701,7 @@
       <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr">
         <is>
-          <t>file_16.xls</t>
+          <t>보장성_상품비교_20260608162103272.xls</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
@@ -4894,7 +4894,7 @@
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr">
         <is>
-          <t>file_16.xls</t>
+          <t>보장성_상품비교_20260608162103272.xls</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
@@ -5087,7 +5087,7 @@
       <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr">
         <is>
-          <t>file_16.xls</t>
+          <t>보장성_상품비교_20260608162103272.xls</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
@@ -5259,7 +5259,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>1,000만원 원</t>
+          <t>1,000만원  원</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -5280,7 +5280,7 @@
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr">
         <is>
-          <t>file_16.xls</t>
+          <t>보장성_상품비교_20260608162103272.xls</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
@@ -5315,7 +5315,7 @@
       </c>
       <c r="W31" t="inlineStr">
         <is>
-          <t>1,000만원 원</t>
+          <t>1,000만원  원</t>
         </is>
       </c>
       <c r="X31" t="inlineStr">
@@ -5427,7 +5427,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>(무) let:play 자녀보험(도담도담)(2601)_6종(100세만기,일반형)</t>
+          <t>(무) let:play 자녀보험(도담도담)(2604)_6종(100세만기,일반형)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -5457,12 +5457,12 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>20,268 원</t>
+          <t>21,502 원</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>17,615 원</t>
+          <t>19,615 원</t>
         </is>
       </c>
       <c r="J32" t="inlineStr"/>
@@ -5473,7 +5473,7 @@
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr">
         <is>
-          <t>file_43.xls</t>
+          <t>장기보장성 비교 공시 (3).xls</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr"/>
@@ -5484,7 +5484,7 @@
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>(무) let:play 자녀보험(도담도담)(2601)_6종(100세만기,일반형)</t>
+          <t>(무) let:play 자녀보험(도담도담)(2604)_6종(100세만기,일반형)</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
@@ -5504,22 +5504,22 @@
       </c>
       <c r="W32" t="inlineStr">
         <is>
-          <t>20,268</t>
+          <t>21,502</t>
         </is>
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>17,615</t>
+          <t>19,615</t>
         </is>
       </c>
       <c r="Y32" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>79.6</t>
         </is>
       </c>
       <c r="Z32" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>72.4</t>
         </is>
       </c>
       <c r="AA32" t="inlineStr"/>
@@ -5556,7 +5556,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>(무) let:play 자녀보험(도담도담)(2601)_9종(100세만기,해약환급금 미지급형Ⅱ)</t>
+          <t>(무) let:play 자녀보험(도담도담)(2604)_9종(100세만기,해약환급금 미지급형Ⅱ)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -5586,12 +5586,12 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>15,890 원</t>
+          <t>17,138 원</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>14,157 원</t>
+          <t>16,064 원</t>
         </is>
       </c>
       <c r="J33" t="inlineStr"/>
@@ -5602,7 +5602,7 @@
       <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr">
         <is>
-          <t>file_43.xls</t>
+          <t>장기보장성 비교 공시 (3).xls</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr"/>
@@ -5613,7 +5613,7 @@
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>(무) let:play 자녀보험(도담도담)(2601)_9종(100세만기,해약환급금 미지급형Ⅱ)</t>
+          <t>(무) let:play 자녀보험(도담도담)(2604)_9종(100세만기,해약환급금 미지급형Ⅱ)</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
@@ -5633,22 +5633,22 @@
       </c>
       <c r="W33" t="inlineStr">
         <is>
-          <t>15,890</t>
+          <t>17,138</t>
         </is>
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>14,157</t>
+          <t>16,064</t>
         </is>
       </c>
       <c r="Y33" t="inlineStr">
         <is>
-          <t>88.5</t>
+          <t>95.5</t>
         </is>
       </c>
       <c r="Z33" t="inlineStr">
         <is>
-          <t>73.5</t>
+          <t>83.4</t>
         </is>
       </c>
       <c r="AA33" t="inlineStr"/>
@@ -5685,7 +5685,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>(무) 내Mom같은 어린이보험2601(1종)(1형)</t>
+          <t>(무) 내Mom같은 어린이보험2604(1종)(1형)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -5731,7 +5731,7 @@
       <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr">
         <is>
-          <t>file_43.xls</t>
+          <t>장기보장성 비교 공시 (3).xls</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr"/>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>(무) 내Mom같은 어린이보험2601(1종)(1형)</t>
+          <t>(무) 내Mom같은 어린이보험2604(1종)(1형)</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
@@ -5814,7 +5814,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>(무) 내Mom같은 어린이보험2601(1종)(3형)</t>
+          <t>(무) 내Mom같은 어린이보험2604(1종)(3형)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -5860,7 +5860,7 @@
       <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr">
         <is>
-          <t>file_43.xls</t>
+          <t>장기보장성 비교 공시 (3).xls</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr"/>
@@ -5871,7 +5871,7 @@
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>(무) 내Mom같은 어린이보험2601(1종)(3형)</t>
+          <t>(무) 내Mom같은 어린이보험2604(1종)(3형)</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
@@ -5943,7 +5943,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>(무) 내Mom같은 어린이보험2601(3종)(1형)</t>
+          <t>(무) 내Mom같은 어린이보험2604(3종)(1형)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -5989,7 +5989,7 @@
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr">
         <is>
-          <t>file_43.xls</t>
+          <t>장기보장성 비교 공시 (3).xls</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr"/>
@@ -6000,7 +6000,7 @@
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>(무) 내Mom같은 어린이보험2601(3종)(1형)</t>
+          <t>(무) 내Mom같은 어린이보험2604(3종)(1형)</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
@@ -6072,7 +6072,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>(무) 내Mom같은 어린이보험2601(3종)(3형)</t>
+          <t>(무) 내Mom같은 어린이보험2604(3종)(3형)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -6118,7 +6118,7 @@
       <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr">
         <is>
-          <t>file_43.xls</t>
+          <t>장기보장성 비교 공시 (3).xls</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr"/>
@@ -6129,7 +6129,7 @@
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>(무) 내Mom같은 어린이보험2601(3종)(3형)</t>
+          <t>(무) 내Mom같은 어린이보험2604(3종)(3형)</t>
         </is>
       </c>
       <c r="T37" t="inlineStr">
@@ -6247,7 +6247,7 @@
       <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr">
         <is>
-          <t>file_16.xls</t>
+          <t>보장성_상품비교_20260608162103272.xls</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
@@ -6440,7 +6440,7 @@
       <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr">
         <is>
-          <t>file_16.xls</t>
+          <t>보장성_상품비교_20260608162103272.xls</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
@@ -6633,7 +6633,7 @@
       <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr">
         <is>
-          <t>file_16.xls</t>
+          <t>보장성_상품비교_20260608162103272.xls</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
@@ -6826,7 +6826,7 @@
       <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr">
         <is>
-          <t>file_16.xls</t>
+          <t>보장성_상품비교_20260608162103272.xls</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
@@ -7019,7 +7019,7 @@
       <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr">
         <is>
-          <t>file_16.xls</t>
+          <t>보장성_상품비교_20260608162103272.xls</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
@@ -7212,7 +7212,7 @@
       <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr">
         <is>
-          <t>file_43.xls</t>
+          <t>장기보장성 비교 공시 (3).xls</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr"/>
@@ -7341,7 +7341,7 @@
       <c r="O44" t="inlineStr"/>
       <c r="P44" t="inlineStr">
         <is>
-          <t>file_43.xls</t>
+          <t>장기보장성 비교 공시 (3).xls</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr"/>
@@ -7470,7 +7470,7 @@
       <c r="O45" t="inlineStr"/>
       <c r="P45" t="inlineStr">
         <is>
-          <t>file_43.xls</t>
+          <t>장기보장성 비교 공시 (3).xls</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr"/>
@@ -7599,7 +7599,7 @@
       <c r="O46" t="inlineStr"/>
       <c r="P46" t="inlineStr">
         <is>
-          <t>file_43.xls</t>
+          <t>장기보장성 비교 공시 (3).xls</t>
         </is>
       </c>
       <c r="Q46" t="inlineStr"/>
@@ -7728,7 +7728,7 @@
       <c r="O47" t="inlineStr"/>
       <c r="P47" t="inlineStr">
         <is>
-          <t>file_43.xls</t>
+          <t>장기보장성 비교 공시 (3).xls</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr"/>
@@ -7857,7 +7857,7 @@
       <c r="O48" t="inlineStr"/>
       <c r="P48" t="inlineStr">
         <is>
-          <t>file_43.xls</t>
+          <t>장기보장성 비교 공시 (3).xls</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr"/>
@@ -7940,7 +7940,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>한화 건강쑥쑥 어린이보험 (무)2601 1종(기본형)</t>
+          <t>한화 건강쑥쑥 어린이보험 (무)2604 1종(기본형)</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -7970,12 +7970,12 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>27,000 원</t>
+          <t>28,700 원</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>23,790 원</t>
+          <t>27,290 원</t>
         </is>
       </c>
       <c r="J49" t="inlineStr"/>
@@ -7986,7 +7986,7 @@
       <c r="O49" t="inlineStr"/>
       <c r="P49" t="inlineStr">
         <is>
-          <t>file_43.xls</t>
+          <t>장기보장성 비교 공시 (3).xls</t>
         </is>
       </c>
       <c r="Q49" t="inlineStr"/>
@@ -7997,7 +7997,7 @@
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>한화 건강쑥쑥 어린이보험 (무)2601 1종(기본형)</t>
+          <t>한화 건강쑥쑥 어린이보험 (무)2604 1종(기본형)</t>
         </is>
       </c>
       <c r="T49" t="inlineStr">
@@ -8017,22 +8017,22 @@
       </c>
       <c r="W49" t="inlineStr">
         <is>
-          <t>27,000</t>
+          <t>28,700</t>
         </is>
       </c>
       <c r="X49" t="inlineStr">
         <is>
-          <t>23,790</t>
+          <t>27,290</t>
         </is>
       </c>
       <c r="Y49" t="inlineStr">
         <is>
-          <t>95.2</t>
+          <t>101.3</t>
         </is>
       </c>
       <c r="Z49" t="inlineStr">
         <is>
-          <t>98.9</t>
+          <t>113.4</t>
         </is>
       </c>
       <c r="AA49" t="inlineStr"/>
@@ -8069,7 +8069,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>한화 건강쑥쑥 어린이보험 (무)2601 2종(납입후50%해약환급금지급형)</t>
+          <t>한화 건강쑥쑥 어린이보험 (무)2604 2종(납입후50%해약환급금지급형)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -8099,12 +8099,12 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>20,340 원</t>
+          <t>20,830 원</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>18,470 원</t>
+          <t>20,190 원</t>
         </is>
       </c>
       <c r="J50" t="inlineStr"/>
@@ -8115,7 +8115,7 @@
       <c r="O50" t="inlineStr"/>
       <c r="P50" t="inlineStr">
         <is>
-          <t>file_43.xls</t>
+          <t>장기보장성 비교 공시 (3).xls</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr"/>
@@ -8126,7 +8126,7 @@
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>한화 건강쑥쑥 어린이보험 (무)2601 2종(납입후50%해약환급금지급형)</t>
+          <t>한화 건강쑥쑥 어린이보험 (무)2604 2종(납입후50%해약환급금지급형)</t>
         </is>
       </c>
       <c r="T50" t="inlineStr">
@@ -8146,22 +8146,22 @@
       </c>
       <c r="W50" t="inlineStr">
         <is>
-          <t>20,340</t>
+          <t>20,830</t>
         </is>
       </c>
       <c r="X50" t="inlineStr">
         <is>
-          <t>18,470</t>
+          <t>20,190</t>
         </is>
       </c>
       <c r="Y50" t="inlineStr">
         <is>
-          <t>108.1</t>
+          <t>110.8</t>
         </is>
       </c>
       <c r="Z50" t="inlineStr">
         <is>
-          <t>112.7</t>
+          <t>123.3</t>
         </is>
       </c>
       <c r="AA50" t="inlineStr"/>
@@ -8244,7 +8244,7 @@
       <c r="O51" t="inlineStr"/>
       <c r="P51" t="inlineStr">
         <is>
-          <t>file_43.xls</t>
+          <t>장기보장성 비교 공시 (3).xls</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr"/>
@@ -8373,7 +8373,7 @@
       <c r="O52" t="inlineStr"/>
       <c r="P52" t="inlineStr">
         <is>
-          <t>file_43.xls</t>
+          <t>장기보장성 비교 공시 (3).xls</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr"/>
@@ -8502,7 +8502,7 @@
       <c r="O53" t="inlineStr"/>
       <c r="P53" t="inlineStr">
         <is>
-          <t>file_43.xls</t>
+          <t>장기보장성 비교 공시 (3).xls</t>
         </is>
       </c>
       <c r="Q53" t="inlineStr"/>
@@ -8631,7 +8631,7 @@
       <c r="O54" t="inlineStr"/>
       <c r="P54" t="inlineStr">
         <is>
-          <t>file_44.xls</t>
+          <t>장기보장성 비교 공시 (4).xls</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr"/>
@@ -8760,7 +8760,7 @@
       <c r="O55" t="inlineStr"/>
       <c r="P55" t="inlineStr">
         <is>
-          <t>file_43.xls</t>
+          <t>장기보장성 비교 공시 (3).xls</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr"/>
@@ -8889,7 +8889,7 @@
       <c r="O56" t="inlineStr"/>
       <c r="P56" t="inlineStr">
         <is>
-          <t>file_44.xls</t>
+          <t>장기보장성 비교 공시 (4).xls</t>
         </is>
       </c>
       <c r="Q56" t="inlineStr"/>
@@ -8972,7 +8972,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>무배당 흥Good 뉴키즈 자녀보험(26.03)_(1종)(해약환급금지급형)</t>
+          <t>무배당 흥Good 뉴키즈 자녀보험(26.05)_(1종)(해약환급금지급형)</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -9002,12 +9002,12 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>68,250 원</t>
+          <t>68,900 원</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>57,980 원</t>
+          <t>58,860 원</t>
         </is>
       </c>
       <c r="J57" t="inlineStr"/>
@@ -9018,7 +9018,7 @@
       <c r="O57" t="inlineStr"/>
       <c r="P57" t="inlineStr">
         <is>
-          <t>file_43.xls</t>
+          <t>장기보장성 비교 공시 (3).xls</t>
         </is>
       </c>
       <c r="Q57" t="inlineStr"/>
@@ -9029,7 +9029,7 @@
       </c>
       <c r="S57" t="inlineStr">
         <is>
-          <t>무배당 흥Good 뉴키즈 자녀보험(26.03)_(1종)(해약환급금지급형)</t>
+          <t>무배당 흥Good 뉴키즈 자녀보험(26.05)_(1종)(해약환급금지급형)</t>
         </is>
       </c>
       <c r="T57" t="inlineStr">
@@ -9049,22 +9049,22 @@
       </c>
       <c r="W57" t="inlineStr">
         <is>
-          <t>68,250</t>
+          <t>68,900</t>
         </is>
       </c>
       <c r="X57" t="inlineStr">
         <is>
-          <t>57,980</t>
+          <t>58,860</t>
         </is>
       </c>
       <c r="Y57" t="inlineStr">
         <is>
-          <t>82.8</t>
+          <t>83.5</t>
         </is>
       </c>
       <c r="Z57" t="inlineStr">
         <is>
-          <t>87.9</t>
+          <t>89.2</t>
         </is>
       </c>
       <c r="AA57" t="inlineStr"/>
@@ -9101,7 +9101,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>무배당 흥Good 뉴키즈 자녀보험(26.03)_(2종)(납입후 해약환급금지급형의 50‰지급형)</t>
+          <t>무배당 흥Good 뉴키즈 자녀보험(26.05)_(2종)(납입후 해약환급금지급형의 50‰지급형)</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -9131,12 +9131,12 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>49,520 원</t>
+          <t>50,030 원</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>41,450 원</t>
+          <t>42,130 원</t>
         </is>
       </c>
       <c r="J58" t="inlineStr"/>
@@ -9147,7 +9147,7 @@
       <c r="O58" t="inlineStr"/>
       <c r="P58" t="inlineStr">
         <is>
-          <t>file_43.xls</t>
+          <t>장기보장성 비교 공시 (3).xls</t>
         </is>
       </c>
       <c r="Q58" t="inlineStr"/>
@@ -9158,7 +9158,7 @@
       </c>
       <c r="S58" t="inlineStr">
         <is>
-          <t>무배당 흥Good 뉴키즈 자녀보험(26.03)_(2종)(납입후 해약환급금지급형의 50‰지급형)</t>
+          <t>무배당 흥Good 뉴키즈 자녀보험(26.05)_(2종)(납입후 해약환급금지급형의 50‰지급형)</t>
         </is>
       </c>
       <c r="T58" t="inlineStr">
@@ -9178,22 +9178,22 @@
       </c>
       <c r="W58" t="inlineStr">
         <is>
-          <t>49,520</t>
+          <t>50,030</t>
         </is>
       </c>
       <c r="X58" t="inlineStr">
         <is>
-          <t>41,450</t>
+          <t>42,130</t>
         </is>
       </c>
       <c r="Y58" t="inlineStr">
         <is>
-          <t>92.3</t>
+          <t>93.2</t>
         </is>
       </c>
       <c r="Z58" t="inlineStr">
         <is>
-          <t>95.4</t>
+          <t>97</t>
         </is>
       </c>
       <c r="AA58" t="inlineStr"/>
@@ -9230,7 +9230,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>무배당 흥Good 뉴키즈 자녀보험(26.03)_(3종)(납입후 표준형환급률 동일지급형)</t>
+          <t>무배당 흥Good 뉴키즈 자녀보험(26.05)_(3종)(납입후 표준형환급률 동일지급형)</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -9260,12 +9260,12 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>56,030 원</t>
+          <t>56,670 원</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>47,880 원</t>
+          <t>48,760 원</t>
         </is>
       </c>
       <c r="J59" t="inlineStr"/>
@@ -9276,7 +9276,7 @@
       <c r="O59" t="inlineStr"/>
       <c r="P59" t="inlineStr">
         <is>
-          <t>file_43.xls</t>
+          <t>장기보장성 비교 공시 (3).xls</t>
         </is>
       </c>
       <c r="Q59" t="inlineStr"/>
@@ -9287,7 +9287,7 @@
       </c>
       <c r="S59" t="inlineStr">
         <is>
-          <t>무배당 흥Good 뉴키즈 자녀보험(26.03)_(3종)(납입후 표준형환급률 동일지급형)</t>
+          <t>무배당 흥Good 뉴키즈 자녀보험(26.05)_(3종)(납입후 표준형환급률 동일지급형)</t>
         </is>
       </c>
       <c r="T59" t="inlineStr">
@@ -9307,22 +9307,22 @@
       </c>
       <c r="W59" t="inlineStr">
         <is>
-          <t>56,030</t>
+          <t>56,670</t>
         </is>
       </c>
       <c r="X59" t="inlineStr">
         <is>
-          <t>47,880</t>
+          <t>48,760</t>
         </is>
       </c>
       <c r="Y59" t="inlineStr">
         <is>
-          <t>93.6</t>
+          <t>94.7</t>
         </is>
       </c>
       <c r="Z59" t="inlineStr">
         <is>
-          <t>99.6</t>
+          <t>101.4</t>
         </is>
       </c>
       <c r="AA59" t="inlineStr"/>

</xml_diff>